<commit_message>
Modified data file Commit
</commit_message>
<xml_diff>
--- a/Jumia_Product_Performance_Dashboard.xlsx
+++ b/Jumia_Product_Performance_Dashboard.xlsx
@@ -8,23 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jndalamia\Documents\DataScience\Jumia Product Performance Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{88DC0FDB-0FB2-4AF3-9A9B-B657F92CBBF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0E3675B-ED25-472B-9AFB-0BFFDA10EB5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="9" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="13" r:id="rId1"/>
     <sheet name="Raw dataset" sheetId="1" r:id="rId2"/>
-    <sheet name="Cleaned data" sheetId="3" r:id="rId3"/>
-    <sheet name="Cleaning log" sheetId="4" r:id="rId4"/>
-    <sheet name="Project Brief" sheetId="2" r:id="rId5"/>
+    <sheet name="Project Brief" sheetId="2" r:id="rId3"/>
+    <sheet name="Cleaned data" sheetId="3" r:id="rId4"/>
+    <sheet name="Cleaning log" sheetId="4" r:id="rId5"/>
     <sheet name="Descriptive Stats" sheetId="6" r:id="rId6"/>
     <sheet name="Enrichment" sheetId="5" r:id="rId7"/>
     <sheet name="Analysis Working" sheetId="7" r:id="rId8"/>
     <sheet name=" Analysis Tables" sheetId="9" r:id="rId9"/>
     <sheet name="Pivot Charts" sheetId="8" r:id="rId10"/>
     <sheet name="Pivot Tables" sheetId="10" r:id="rId11"/>
-    <sheet name="Exception" sheetId="11" r:id="rId12"/>
+    <sheet name="Exceptions" sheetId="11" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Analysis Working'!$A$1:$J$113</definedName>
@@ -35,8 +35,8 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId13"/>
-    <pivotCache cacheId="1" r:id="rId14"/>
+    <pivotCache cacheId="4" r:id="rId13"/>
+    <pivotCache cacheId="5" r:id="rId14"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -2427,9 +2427,6 @@
     <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2440,6 +2437,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -14275,313 +14275,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0900-000001000000}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8">
-  <location ref="A20:B24" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="9" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="3"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="9"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Average of Rating" fld="5" subtotal="average" baseField="9" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="3">
-    <chartFormat chart="0" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="2" format="3" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="7" format="5" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0900-000006000000}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
-  <location ref="A2:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="9" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="3"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="4">
-        <item x="2"/>
-        <item x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="8"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Average of Review" fld="4" subtotal="average" baseField="8" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="4">
-    <chartFormat chart="0" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="2" format="5" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="4" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="10" format="7" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0900-000005000000}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A28:E35" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="9" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="3"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="7"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="8"/>
-  </colFields>
-  <colItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of Product" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0900-000000000000}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0900-000000000000}" name="PivotTable3" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
   <location ref="A10:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
@@ -14688,8 +14382,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0900-000004000000}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="4" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0900-000004000000}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="4" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A38:B48" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" measureFilter="1" sortType="descending" defaultSubtotal="0">
@@ -15022,8 +14716,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0900-000003000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="4" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0900-000003000000}" name="PivotTable9" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="4" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A75:B85" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" measureFilter="1" sortType="descending" defaultSubtotal="0">
@@ -15365,8 +15059,221 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0900-000002000000}" name="PivotTable6" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="4" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0900-000001000000}" name="PivotTable4" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8">
+  <location ref="A20:B24" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="9" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="3"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="9"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average of Rating" fld="5" subtotal="average" baseField="9" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="3">
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="7" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0900-000006000000}" name="PivotTable2" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
+  <location ref="A2:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="9" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="3"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="2"/>
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="8"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average of Review" fld="4" subtotal="average" baseField="8" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="4">
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="4" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="10" format="7" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0900-000002000000}" name="PivotTable6" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="4" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A59:B69" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" measureFilter="1" sortType="descending" defaultSubtotal="0">
@@ -15688,6 +15595,99 @@
       </autoFilter>
     </filter>
   </filters>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0900-000005000000}" name="PivotTable5" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="4" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A28:E35" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="9" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="3"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="8"/>
+  </colFields>
+  <colItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Product" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
       <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
@@ -16066,140 +16066,140 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="26" t="s">
         <v>494</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="28"/>
-      <c r="P1" s="28"/>
-      <c r="Q1" s="28"/>
-      <c r="R1" s="28"/>
-      <c r="S1" s="28"/>
-      <c r="T1" s="28"/>
-      <c r="U1" s="28"/>
-      <c r="V1" s="28"/>
-      <c r="W1" s="28"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
+      <c r="T1" s="27"/>
+      <c r="U1" s="27"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="27"/>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A2" s="28"/>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
-      <c r="L2" s="28"/>
-      <c r="M2" s="28"/>
-      <c r="N2" s="28"/>
-      <c r="O2" s="28"/>
-      <c r="P2" s="28"/>
-      <c r="Q2" s="28"/>
-      <c r="R2" s="28"/>
-      <c r="S2" s="28"/>
-      <c r="T2" s="28"/>
-      <c r="U2" s="28"/>
-      <c r="V2" s="28"/>
-      <c r="W2" s="28"/>
+      <c r="A2" s="27"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="27"/>
+      <c r="P2" s="27"/>
+      <c r="Q2" s="27"/>
+      <c r="R2" s="27"/>
+      <c r="S2" s="27"/>
+      <c r="T2" s="27"/>
+      <c r="U2" s="27"/>
+      <c r="V2" s="27"/>
+      <c r="W2" s="27"/>
     </row>
     <row r="3" spans="1:23" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="28" t="s">
         <v>495</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
-      <c r="M3" s="29"/>
-      <c r="N3" s="29"/>
-      <c r="O3" s="29"/>
-      <c r="P3" s="29"/>
-      <c r="Q3" s="29"/>
-      <c r="R3" s="29"/>
-      <c r="S3" s="29"/>
-      <c r="T3" s="29"/>
-      <c r="U3" s="29"/>
-      <c r="V3" s="29"/>
-      <c r="W3" s="29"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="28"/>
+      <c r="P3" s="28"/>
+      <c r="Q3" s="28"/>
+      <c r="R3" s="28"/>
+      <c r="S3" s="28"/>
+      <c r="T3" s="28"/>
+      <c r="U3" s="28"/>
+      <c r="V3" s="28"/>
+      <c r="W3" s="28"/>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="29" t="s">
         <v>500</v>
       </c>
-      <c r="B9" s="25"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
-      <c r="H9" s="25" t="s">
+      <c r="B9" s="29"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="H9" s="29" t="s">
         <v>501</v>
       </c>
-      <c r="I9" s="25"/>
-      <c r="J9" s="25"/>
-      <c r="K9" s="25"/>
-      <c r="L9" s="25"/>
-      <c r="M9" s="25"/>
-      <c r="O9" s="25" t="s">
+      <c r="I9" s="29"/>
+      <c r="J9" s="29"/>
+      <c r="K9" s="29"/>
+      <c r="L9" s="29"/>
+      <c r="M9" s="29"/>
+      <c r="O9" s="29" t="s">
         <v>502</v>
       </c>
-      <c r="P9" s="25"/>
-      <c r="Q9" s="25"/>
-      <c r="R9" s="25"/>
-      <c r="S9" s="25"/>
-      <c r="T9" s="25"/>
+      <c r="P9" s="29"/>
+      <c r="Q9" s="29"/>
+      <c r="R9" s="29"/>
+      <c r="S9" s="29"/>
+      <c r="T9" s="29"/>
     </row>
     <row r="10" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="26" t="s">
+      <c r="A10" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
       <c r="F10" s="20" t="s">
         <v>503</v>
       </c>
       <c r="G10" s="19"/>
-      <c r="H10" s="26" t="s">
+      <c r="H10" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="I10" s="26"/>
-      <c r="J10" s="26"/>
-      <c r="K10" s="26"/>
-      <c r="L10" s="26"/>
+      <c r="I10" s="25"/>
+      <c r="J10" s="25"/>
+      <c r="K10" s="25"/>
+      <c r="L10" s="25"/>
       <c r="M10" s="20" t="s">
         <v>351</v>
       </c>
       <c r="N10" s="19"/>
-      <c r="O10" s="26" t="s">
+      <c r="O10" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="P10" s="26"/>
-      <c r="Q10" s="26"/>
-      <c r="R10" s="26"/>
-      <c r="S10" s="26"/>
+      <c r="P10" s="25"/>
+      <c r="Q10" s="25"/>
+      <c r="R10" s="25"/>
+      <c r="S10" s="25"/>
       <c r="T10" s="20" t="s">
         <v>3</v>
       </c>
@@ -16526,28 +16526,6 @@
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="H13:L13"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A17:E17"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="H15:L15"/>
-    <mergeCell ref="H16:L16"/>
-    <mergeCell ref="H17:L17"/>
-    <mergeCell ref="H18:L18"/>
-    <mergeCell ref="H19:L19"/>
-    <mergeCell ref="A1:W2"/>
-    <mergeCell ref="A3:W3"/>
-    <mergeCell ref="H10:L10"/>
-    <mergeCell ref="H11:L11"/>
-    <mergeCell ref="H12:L12"/>
     <mergeCell ref="O19:S19"/>
     <mergeCell ref="O20:S20"/>
     <mergeCell ref="A9:F9"/>
@@ -16564,6 +16542,28 @@
     <mergeCell ref="O17:S17"/>
     <mergeCell ref="O18:S18"/>
     <mergeCell ref="H14:L14"/>
+    <mergeCell ref="A1:W2"/>
+    <mergeCell ref="A3:W3"/>
+    <mergeCell ref="H10:L10"/>
+    <mergeCell ref="H11:L11"/>
+    <mergeCell ref="H12:L12"/>
+    <mergeCell ref="H13:L13"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="H15:L15"/>
+    <mergeCell ref="H16:L16"/>
+    <mergeCell ref="H17:L17"/>
+    <mergeCell ref="H18:L18"/>
+    <mergeCell ref="H19:L19"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A15:E15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -20839,6 +20839,165 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr>
+    <tabColor theme="2" tint="-0.249977111117893"/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="101.7109375" customWidth="1"/>
+    <col min="3" max="3" width="37.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>350</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor theme="3" tint="0.59999389629810485"/>
@@ -23121,7 +23280,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="1" tint="0.34998626667073579"/>
@@ -23651,165 +23810,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr>
-    <tabColor theme="2" tint="-0.249977111117893"/>
-  </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="23.42578125" customWidth="1"/>
-    <col min="2" max="2" width="101.7109375" customWidth="1"/>
-    <col min="3" max="3" width="37.28515625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>323</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>324</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>326</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>330</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>332</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>336</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>339</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>340</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>342</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>344</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>344</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>347</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>344</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>344</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>350</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>